<commit_message>
Update model outputs 2026-06-10 07:24:44
</commit_message>
<xml_diff>
--- a/files/ANZ_upcoming_projections.xlsx
+++ b/files/ANZ_upcoming_projections.xlsx
@@ -65,28 +65,28 @@
     <t xml:space="preserve">1H</t>
   </si>
   <si>
+    <t xml:space="preserve">Northern Mystics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waikato Bay of Plenty Magic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northern Stars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Pulse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Steel</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mainland Tactix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern Mystics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waikato Bay of Plenty Magic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Pulse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern Stars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern Steel</t>
   </si>
 </sst>
 </file>
@@ -423,8 +423,8 @@
   <cols>
     <col min="1" max="1" width="11.2056266178838" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="27.709999474506" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="16.7099996885961" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="27.709999474506" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.704168823845" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.8703495591654" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="20.5350725004471" hidden="0" customWidth="1"/>
@@ -491,7 +491,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -503,45 +503,45 @@
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>1.16</v>
+        <v>-7.06</v>
       </c>
       <c r="F2" t="n">
-        <v>52.21</v>
+        <v>50.16</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H2" t="n">
-        <v>1.02</v>
+        <v>-7.11</v>
       </c>
       <c r="I2" t="n">
-        <v>49.96</v>
+        <v>49.09</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.09</v>
+        <v>1.73</v>
       </c>
       <c r="L2" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.45</v>
+        <v>0.16</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.15</v>
+        <v>0.16</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7</v>
+        <v>-6.9</v>
       </c>
       <c r="P2" t="n">
-        <v>52.06</v>
+        <v>50.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -553,45 +553,45 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>0.59</v>
+        <v>-3.55</v>
       </c>
       <c r="F3" t="n">
-        <v>26.1</v>
+        <v>25.06</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H3" t="n">
-        <v>0.52</v>
+        <v>-3.58</v>
       </c>
       <c r="I3" t="n">
-        <v>24.98</v>
+        <v>24.53</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.09</v>
+        <v>1.73</v>
       </c>
       <c r="L3" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.23</v>
+        <v>0.08</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.07</v>
+        <v>0.08</v>
       </c>
       <c r="O3" t="n">
-        <v>0.36</v>
+        <v>-3.47</v>
       </c>
       <c r="P3" t="n">
-        <v>26.03</v>
+        <v>25.14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -603,45 +603,45 @@
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>2.26</v>
+        <v>-13.95</v>
       </c>
       <c r="F4" t="n">
-        <v>104.64</v>
+        <v>100.53</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H4" t="n">
-        <v>1.99</v>
+        <v>-14.05</v>
       </c>
       <c r="I4" t="n">
-        <v>100.13</v>
+        <v>98.4</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.09</v>
+        <v>1.73</v>
       </c>
       <c r="L4" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.9</v>
+        <v>0.33</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.3</v>
+        <v>0.31</v>
       </c>
       <c r="O4" t="n">
-        <v>1.36</v>
+        <v>-13.63</v>
       </c>
       <c r="P4" t="n">
-        <v>104.35</v>
+        <v>100.84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -653,45 +653,45 @@
         <v>22</v>
       </c>
       <c r="E5" t="n">
-        <v>2.77</v>
+        <v>-2.79</v>
       </c>
       <c r="F5" t="n">
-        <v>49.23</v>
+        <v>56.85</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H5" t="n">
-        <v>2.79</v>
+        <v>-2.48</v>
       </c>
       <c r="I5" t="n">
-        <v>48.86</v>
+        <v>53.56</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1.01</v>
+        <v>1.8</v>
       </c>
       <c r="L5" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.03</v>
+        <v>-0.11</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.1</v>
+        <v>0.25</v>
       </c>
       <c r="O5" t="n">
-        <v>2.74</v>
+        <v>-2.9</v>
       </c>
       <c r="P5" t="n">
-        <v>49.13</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
@@ -703,45 +703,45 @@
         <v>22</v>
       </c>
       <c r="E6" t="n">
-        <v>1.41</v>
+        <v>-1.41</v>
       </c>
       <c r="F6" t="n">
-        <v>24.61</v>
+        <v>28.4</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H6" t="n">
-        <v>1.42</v>
+        <v>-1.25</v>
       </c>
       <c r="I6" t="n">
-        <v>24.43</v>
+        <v>26.76</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>1.01</v>
+        <v>1.8</v>
       </c>
       <c r="L6" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.02</v>
+        <v>-0.05</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.05</v>
+        <v>0.12</v>
       </c>
       <c r="O6" t="n">
-        <v>1.4</v>
+        <v>-1.46</v>
       </c>
       <c r="P6" t="n">
-        <v>24.56</v>
+        <v>28.53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46179</v>
+        <v>46186</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
@@ -753,45 +753,45 @@
         <v>22</v>
       </c>
       <c r="E7" t="n">
-        <v>5.41</v>
+        <v>-5.52</v>
       </c>
       <c r="F7" t="n">
-        <v>98.67</v>
+        <v>113.96</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H7" t="n">
-        <v>5.46</v>
+        <v>-4.91</v>
       </c>
       <c r="I7" t="n">
-        <v>97.92</v>
+        <v>107.35</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1.01</v>
+        <v>1.8</v>
       </c>
       <c r="L7" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.06</v>
+        <v>-0.21</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.2</v>
+        <v>0.49</v>
       </c>
       <c r="O7" t="n">
-        <v>5.35</v>
+        <v>-5.73</v>
       </c>
       <c r="P7" t="n">
-        <v>98.47</v>
+        <v>114.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46180</v>
+        <v>46187</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -803,45 +803,45 @@
         <v>24</v>
       </c>
       <c r="E8" t="n">
-        <v>1.84</v>
+        <v>-1.56</v>
       </c>
       <c r="F8" t="n">
-        <v>57.68</v>
+        <v>51.15</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H8" t="n">
-        <v>1.52</v>
+        <v>-1.53</v>
       </c>
       <c r="I8" t="n">
-        <v>57.32</v>
+        <v>52.76</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1.14</v>
+        <v>1.67</v>
       </c>
       <c r="L8" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1</v>
+        <v>-0.07</v>
       </c>
       <c r="N8" t="n">
-        <v>0.21</v>
+        <v>-0.47</v>
       </c>
       <c r="O8" t="n">
-        <v>1.94</v>
+        <v>-1.63</v>
       </c>
       <c r="P8" t="n">
-        <v>57.89</v>
+        <v>50.68</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46180</v>
+        <v>46187</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
@@ -853,45 +853,45 @@
         <v>24</v>
       </c>
       <c r="E9" t="n">
-        <v>0.93</v>
+        <v>-0.78</v>
       </c>
       <c r="F9" t="n">
-        <v>28.84</v>
+        <v>25.56</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H9" t="n">
-        <v>0.78</v>
+        <v>-0.77</v>
       </c>
       <c r="I9" t="n">
-        <v>28.66</v>
+        <v>26.36</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1.14</v>
+        <v>1.67</v>
       </c>
       <c r="L9" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M9" t="n">
-        <v>0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1</v>
+        <v>-0.24</v>
       </c>
       <c r="O9" t="n">
-        <v>0.99</v>
+        <v>-0.82</v>
       </c>
       <c r="P9" t="n">
-        <v>28.94</v>
+        <v>25.32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46180</v>
+        <v>46187</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
@@ -903,40 +903,40 @@
         <v>24</v>
       </c>
       <c r="E10" t="n">
-        <v>3.59</v>
+        <v>-3.07</v>
       </c>
       <c r="F10" t="n">
-        <v>115.61</v>
+        <v>102.53</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.3</v>
+        <v>-0.22</v>
       </c>
       <c r="H10" t="n">
-        <v>2.98</v>
+        <v>-3.02</v>
       </c>
       <c r="I10" t="n">
-        <v>114.89</v>
+        <v>105.75</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1.14</v>
+        <v>1.67</v>
       </c>
       <c r="L10" t="n">
-        <v>1.22</v>
+        <v>1.72</v>
       </c>
       <c r="M10" t="n">
-        <v>0.21</v>
+        <v>-0.14</v>
       </c>
       <c r="N10" t="n">
-        <v>0.41</v>
+        <v>-0.95</v>
       </c>
       <c r="O10" t="n">
-        <v>3.8</v>
+        <v>-3.22</v>
       </c>
       <c r="P10" t="n">
-        <v>116.02</v>
+        <v>101.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-06-20 17:01:28
</commit_message>
<xml_diff>
--- a/files/ANZ_upcoming_projections.xlsx
+++ b/files/ANZ_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">game_date</t>
   </si>
@@ -65,28 +65,16 @@
     <t xml:space="preserve">1H</t>
   </si>
   <si>
-    <t xml:space="preserve">Northern Mystics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waikato Bay of Plenty Magic</t>
+    <t xml:space="preserve">Southern Steel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mainland Tactix</t>
   </si>
   <si>
     <t xml:space="preserve">1Q</t>
   </si>
   <si>
     <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern Stars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Pulse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern Steel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mainland Tactix</t>
   </si>
 </sst>
 </file>
@@ -423,8 +411,8 @@
   <cols>
     <col min="1" max="1" width="11.2056266178838" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="27.709999474506" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.7099997275216" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.7099997080589" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.704168823845" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.8703495591654" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="20.5350725004471" hidden="0" customWidth="1"/>
@@ -491,7 +479,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46186</v>
+        <v>46194</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -503,45 +491,45 @@
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>-7.06</v>
+        <v>-1.44</v>
       </c>
       <c r="F2" t="n">
-        <v>50.16</v>
+        <v>52.11</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.22</v>
+        <v>-0.25</v>
       </c>
       <c r="H2" t="n">
-        <v>-7.11</v>
+        <v>-1.42</v>
       </c>
       <c r="I2" t="n">
-        <v>49.09</v>
+        <v>53.45</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L2" t="n">
-        <v>1.72</v>
+        <v>1.75</v>
       </c>
       <c r="M2" t="n">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
       <c r="N2" t="n">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>-6.9</v>
+        <v>-1.4</v>
       </c>
       <c r="P2" t="n">
-        <v>50.31</v>
+        <v>52.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46186</v>
+        <v>46194</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -553,45 +541,45 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>-3.55</v>
+        <v>-0.74</v>
       </c>
       <c r="F3" t="n">
-        <v>25.06</v>
+        <v>26.04</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.22</v>
+        <v>-0.25</v>
       </c>
       <c r="H3" t="n">
-        <v>-3.58</v>
+        <v>-0.73</v>
       </c>
       <c r="I3" t="n">
-        <v>24.53</v>
+        <v>26.71</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L3" t="n">
-        <v>1.72</v>
+        <v>1.75</v>
       </c>
       <c r="M3" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="N3" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>-3.47</v>
+        <v>-0.72</v>
       </c>
       <c r="P3" t="n">
-        <v>25.14</v>
+        <v>26.04</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46186</v>
+        <v>46194</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -603,340 +591,40 @@
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>-13.95</v>
+        <v>-2.85</v>
       </c>
       <c r="F4" t="n">
-        <v>100.53</v>
+        <v>104.45</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.22</v>
+        <v>-0.25</v>
       </c>
       <c r="H4" t="n">
-        <v>-14.05</v>
+        <v>-2.82</v>
       </c>
       <c r="I4" t="n">
-        <v>98.4</v>
+        <v>107.14</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L4" t="n">
-        <v>1.72</v>
+        <v>1.75</v>
       </c>
       <c r="M4" t="n">
-        <v>0.33</v>
+        <v>0.08</v>
       </c>
       <c r="N4" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>-13.63</v>
+        <v>-2.77</v>
       </c>
       <c r="P4" t="n">
-        <v>100.84</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-2.79</v>
-      </c>
-      <c r="F5" t="n">
-        <v>56.85</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-2.48</v>
-      </c>
-      <c r="I5" t="n">
-        <v>53.56</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O5" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="P5" t="n">
-        <v>57.1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-1.41</v>
-      </c>
-      <c r="F6" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-1.25</v>
-      </c>
-      <c r="I6" t="n">
-        <v>26.76</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="O6" t="n">
-        <v>-1.46</v>
-      </c>
-      <c r="P6" t="n">
-        <v>28.53</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="n">
-        <v>-5.52</v>
-      </c>
-      <c r="F7" t="n">
-        <v>113.96</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-4.91</v>
-      </c>
-      <c r="I7" t="n">
-        <v>107.35</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-0.21</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="O7" t="n">
-        <v>-5.73</v>
-      </c>
-      <c r="P7" t="n">
-        <v>114.45</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-1.56</v>
-      </c>
-      <c r="F8" t="n">
-        <v>51.15</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-1.53</v>
-      </c>
-      <c r="I8" t="n">
-        <v>52.76</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M8" t="n">
-        <v>-0.07</v>
-      </c>
-      <c r="N8" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="O8" t="n">
-        <v>-1.63</v>
-      </c>
-      <c r="P8" t="n">
-        <v>50.68</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-0.78</v>
-      </c>
-      <c r="F9" t="n">
-        <v>25.56</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="I9" t="n">
-        <v>26.36</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M9" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="N9" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="O9" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="P9" t="n">
-        <v>25.32</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-3.07</v>
-      </c>
-      <c r="F10" t="n">
-        <v>102.53</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="H10" t="n">
-        <v>-3.02</v>
-      </c>
-      <c r="I10" t="n">
-        <v>105.75</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-0.14</v>
-      </c>
-      <c r="N10" t="n">
-        <v>-0.95</v>
-      </c>
-      <c r="O10" t="n">
-        <v>-3.22</v>
-      </c>
-      <c r="P10" t="n">
-        <v>101.58</v>
+        <v>104.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-06-26 09:39:09
</commit_message>
<xml_diff>
--- a/files/ANZ_upcoming_projections.xlsx
+++ b/files/ANZ_upcoming_projections.xlsx
@@ -65,10 +65,10 @@
     <t xml:space="preserve">1H</t>
   </si>
   <si>
+    <t xml:space="preserve">Northern Mystics</t>
+  </si>
+  <si>
     <t xml:space="preserve">Southern Steel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mainland Tactix</t>
   </si>
   <si>
     <t xml:space="preserve">1Q</t>
@@ -411,8 +411,8 @@
   <cols>
     <col min="1" max="1" width="11.2056266178838" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="14.7099997275216" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="15.7099997080589" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14.7099997275216" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.704168823845" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.8703495591654" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="20.5350725004471" hidden="0" customWidth="1"/>
@@ -479,7 +479,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -491,45 +491,45 @@
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>-1.44</v>
+        <v>-1.64</v>
       </c>
       <c r="F2" t="n">
-        <v>52.11</v>
+        <v>53.93</v>
       </c>
       <c r="G2" t="n">
         <v>-0.25</v>
       </c>
       <c r="H2" t="n">
-        <v>-1.42</v>
+        <v>-1.63</v>
       </c>
       <c r="I2" t="n">
-        <v>53.45</v>
+        <v>56.25</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.69</v>
+        <v>1.73</v>
       </c>
       <c r="L2" t="n">
         <v>1.75</v>
       </c>
       <c r="M2" t="n">
-        <v>0.04</v>
+        <v>-0.17</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>-1.4</v>
+        <v>-1.81</v>
       </c>
       <c r="P2" t="n">
-        <v>52.11</v>
+        <v>53.92</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -541,45 +541,45 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.74</v>
+        <v>-0.84</v>
       </c>
       <c r="F3" t="n">
-        <v>26.04</v>
+        <v>26.95</v>
       </c>
       <c r="G3" t="n">
         <v>-0.25</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.73</v>
+        <v>-0.83</v>
       </c>
       <c r="I3" t="n">
-        <v>26.71</v>
+        <v>28.11</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.69</v>
+        <v>1.73</v>
       </c>
       <c r="L3" t="n">
         <v>1.75</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02</v>
+        <v>-0.09</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.72</v>
+        <v>-0.93</v>
       </c>
       <c r="P3" t="n">
-        <v>26.04</v>
+        <v>26.95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46194</v>
+        <v>46200</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -591,40 +591,40 @@
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>-2.85</v>
+        <v>-3.25</v>
       </c>
       <c r="F4" t="n">
-        <v>104.45</v>
+        <v>108.09</v>
       </c>
       <c r="G4" t="n">
         <v>-0.25</v>
       </c>
       <c r="H4" t="n">
-        <v>-2.82</v>
+        <v>-3.22</v>
       </c>
       <c r="I4" t="n">
-        <v>107.14</v>
+        <v>112.74</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.69</v>
+        <v>1.73</v>
       </c>
       <c r="L4" t="n">
         <v>1.75</v>
       </c>
       <c r="M4" t="n">
-        <v>0.08</v>
+        <v>-0.34</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="O4" t="n">
-        <v>-2.77</v>
+        <v>-3.59</v>
       </c>
       <c r="P4" t="n">
-        <v>104.45</v>
+        <v>108.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-03 15:38:09
</commit_message>
<xml_diff>
--- a/files/ANZ_upcoming_projections.xlsx
+++ b/files/ANZ_upcoming_projections.xlsx
@@ -65,10 +65,10 @@
     <t xml:space="preserve">1H</t>
   </si>
   <si>
-    <t xml:space="preserve">Northern Mystics</t>
-  </si>
-  <si>
     <t xml:space="preserve">Southern Steel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mainland Tactix</t>
   </si>
   <si>
     <t xml:space="preserve">1Q</t>
@@ -411,8 +411,8 @@
   <cols>
     <col min="1" max="1" width="11.2056266178838" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="14.7099997275216" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.7099997275216" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.7099997080589" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.704168823845" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.8703495591654" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="20.5350725004471" hidden="0" customWidth="1"/>
@@ -479,7 +479,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46200</v>
+        <v>46194</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -491,45 +491,45 @@
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>-1.64</v>
+        <v>-1.44</v>
       </c>
       <c r="F2" t="n">
-        <v>53.93</v>
+        <v>52.11</v>
       </c>
       <c r="G2" t="n">
         <v>-0.25</v>
       </c>
       <c r="H2" t="n">
-        <v>-1.63</v>
+        <v>-1.42</v>
       </c>
       <c r="I2" t="n">
-        <v>56.25</v>
+        <v>53.45</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L2" t="n">
         <v>1.75</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.17</v>
+        <v>0.04</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>-1.81</v>
+        <v>-1.4</v>
       </c>
       <c r="P2" t="n">
-        <v>53.92</v>
+        <v>52.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46200</v>
+        <v>46194</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -541,45 +541,45 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.84</v>
+        <v>-0.74</v>
       </c>
       <c r="F3" t="n">
-        <v>26.95</v>
+        <v>26.04</v>
       </c>
       <c r="G3" t="n">
         <v>-0.25</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.83</v>
+        <v>-0.73</v>
       </c>
       <c r="I3" t="n">
-        <v>28.11</v>
+        <v>26.71</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L3" t="n">
         <v>1.75</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.09</v>
+        <v>0.02</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.93</v>
+        <v>-0.72</v>
       </c>
       <c r="P3" t="n">
-        <v>26.95</v>
+        <v>26.04</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46200</v>
+        <v>46194</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -591,40 +591,40 @@
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>-3.25</v>
+        <v>-2.85</v>
       </c>
       <c r="F4" t="n">
-        <v>108.09</v>
+        <v>104.45</v>
       </c>
       <c r="G4" t="n">
         <v>-0.25</v>
       </c>
       <c r="H4" t="n">
-        <v>-3.22</v>
+        <v>-2.82</v>
       </c>
       <c r="I4" t="n">
-        <v>112.74</v>
+        <v>107.14</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="L4" t="n">
         <v>1.75</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.34</v>
+        <v>0.08</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>-3.59</v>
+        <v>-2.77</v>
       </c>
       <c r="P4" t="n">
-        <v>108.09</v>
+        <v>104.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>